<commit_message>
Summative: match xlsx template exactly, drop password protection, add Word export
- build_summative_sheet now reproduces summative_sample.xlsx exactly:
  org/title sizes 13/12, assessor & mean-deviation lines above the table,
  header at row 14 (repeat row), candidate rows from 15, 3-line signatory
  block. Verified cell-for-cell against the template.
- Removed sheet password protection — the sheet is filled in by hand.
- New summative_word.py: build_summative_per_unit_docx() renders the same
  template as .docx (TNR, blue title, grey-shaded bordered table, signatory
  block). python-docx added to requirements.
- Summative view gets an Excel/Word format toggle; _gen_summative_zip takes
  a fmt arg and the cache key includes it.
- Regenerated summative_sample.xlsx (now unprotected).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/summative_sample.xlsx
+++ b/summative_sample.xlsx
@@ -181,7 +181,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -213,10 +213,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1006,9 +1002,9 @@
           <t>ACHIENG JOYCE ATIENO</t>
         </is>
       </c>
-      <c r="D15" s="18" t="n"/>
-      <c r="E15" s="18" t="n"/>
-      <c r="F15" s="18" t="n"/>
+      <c r="D15" s="16" t="n"/>
+      <c r="E15" s="16" t="n"/>
+      <c r="F15" s="16" t="n"/>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="16" t="n">
@@ -1024,9 +1020,9 @@
           <t>BETT KIPRONO JAMES</t>
         </is>
       </c>
-      <c r="D16" s="18" t="n"/>
-      <c r="E16" s="18" t="n"/>
-      <c r="F16" s="18" t="n"/>
+      <c r="D16" s="16" t="n"/>
+      <c r="E16" s="16" t="n"/>
+      <c r="F16" s="16" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="16" t="n">
@@ -1042,9 +1038,9 @@
           <t>CHEBET FAITH JELIMO</t>
         </is>
       </c>
-      <c r="D17" s="18" t="n"/>
-      <c r="E17" s="18" t="n"/>
-      <c r="F17" s="18" t="n"/>
+      <c r="D17" s="16" t="n"/>
+      <c r="E17" s="16" t="n"/>
+      <c r="F17" s="16" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="16" t="n">
@@ -1060,9 +1056,9 @@
           <t>GITAU DAVID MWANGI</t>
         </is>
       </c>
-      <c r="D18" s="18" t="n"/>
-      <c r="E18" s="18" t="n"/>
-      <c r="F18" s="18" t="n"/>
+      <c r="D18" s="16" t="n"/>
+      <c r="E18" s="16" t="n"/>
+      <c r="F18" s="16" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="16" t="n">
@@ -1078,9 +1074,9 @@
           <t>HASSAN IBRAHIM OMAR</t>
         </is>
       </c>
-      <c r="D19" s="18" t="n"/>
-      <c r="E19" s="18" t="n"/>
-      <c r="F19" s="18" t="n"/>
+      <c r="D19" s="16" t="n"/>
+      <c r="E19" s="16" t="n"/>
+      <c r="F19" s="16" t="n"/>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="16" t="n">
@@ -1096,9 +1092,9 @@
           <t>KAMAU WANJIKU GRACE</t>
         </is>
       </c>
-      <c r="D20" s="18" t="n"/>
-      <c r="E20" s="18" t="n"/>
-      <c r="F20" s="18" t="n"/>
+      <c r="D20" s="16" t="n"/>
+      <c r="E20" s="16" t="n"/>
+      <c r="F20" s="16" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="16" t="n">
@@ -1114,9 +1110,9 @@
           <t>LANGAT KIPCHOGE ENOCH</t>
         </is>
       </c>
-      <c r="D21" s="18" t="n"/>
-      <c r="E21" s="18" t="n"/>
-      <c r="F21" s="18" t="n"/>
+      <c r="D21" s="16" t="n"/>
+      <c r="E21" s="16" t="n"/>
+      <c r="F21" s="16" t="n"/>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="16" t="n">
@@ -1132,9 +1128,9 @@
           <t>MUTUA STEPHEN NDULI</t>
         </is>
       </c>
-      <c r="D22" s="18" t="n"/>
-      <c r="E22" s="18" t="n"/>
-      <c r="F22" s="18" t="n"/>
+      <c r="D22" s="16" t="n"/>
+      <c r="E22" s="16" t="n"/>
+      <c r="F22" s="16" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1"/>
     <row r="24" ht="22" customHeight="1">
@@ -1306,7 +1302,6 @@
       <c r="F26" s="14" t="n"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CC1B"/>
   <mergeCells count="19">
     <mergeCell ref="A12:F12"/>
     <mergeCell ref="D7:F7"/>

</xml_diff>